<commit_message>
fixed class for Ambra Ravara
</commit_message>
<xml_diff>
--- a/static/results/2026_territoriali_risultati.xlsx
+++ b/static/results/2026_territoriali_risultati.xlsx
@@ -10699,7 +10699,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:X1120"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.11"/>
@@ -24307,7 +24307,7 @@
         <v>959</v>
       </c>
       <c r="M184" s="0" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N184" s="0" t="s">
         <v>960</v>

</xml_diff>